<commit_message>
One percent-change panel per scenario, on their own charts tab
The combined chart puts sixteen series on one pair of axes, which shows which
scenarios move together but buries any single line. These are the same data one
panel at a time, referencing the 'percent change' grid rather than copying it, so
the two cannot disagree.

Panels autoscale individually -- a common scale would flatten the small movers
against the reservation runs -- but each axis is forced to span zero, so "above
or below central" is never an artefact of where the axis starts.

Central is skipped: its own percent-change column is zero by construction.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018pSRAMaSP6de6HFGRLmysE
</commit_message>
<xml_diff>
--- a/output/domestic_price_summary.xlsx
+++ b/output/domestic_price_summary.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="levels" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="percent change" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="charts" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -773,6 +774,1077 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>SC  ·  W-M L-M  ·  No imports  ·  Netback</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'percent change'!J1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'percent change'!$A$2:$A$27</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'percent change'!$J$2:$J$27</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Year</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="71.50952316672017"/>
+          <min val="0"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>% vs central</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart11.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>SC  ·  W-M L-M  ·  GSOO exp  ·  Netback</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'percent change'!K1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'percent change'!$A$2:$A$27</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'percent change'!$K$2:$K$27</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Year</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="7.709110301617583"/>
+          <min val="-0.7561469943685784"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>% vs central</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart12.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>SC  ·  W-M L-M  ·  Res20%  ·  Netback</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'percent change'!L1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'percent change'!$A$2:$A$27</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'percent change'!$L$2:$L$27</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Year</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="22.5482665569533"/>
+          <min val="-0.766637447044205"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>% vs central</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart13.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>SC  ·  W-M L-M  ·  DC series NSW  ·  Netback</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'percent change'!M1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'percent change'!$A$2:$A$27</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'percent change'!$M$2:$M$27</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Year</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="2.916091695439627"/>
+          <min val="-1.598763468300524"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>% vs central</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart14.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>SC  ·  W-H L-M  ·  DC series NSW  ·  Netback</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'percent change'!N1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'percent change'!$A$2:$A$27</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'percent change'!$N$2:$N$27</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Year</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="9.792466076806662"/>
+          <min val="-2.485651486958362"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>% vs central</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart15.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>SC  ·  W-M L-M  ·  DC series NSW  ·  No imports  ·  Netback</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'percent change'!O1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'percent change'!$A$2:$A$27</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'percent change'!$O$2:$O$27</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Year</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="84.8294911052738"/>
+          <min val="0"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>% vs central</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart16.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>SC  ·  W-M L-M  ·  Res20%+contract  ·  Netback</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'percent change'!P1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'percent change'!$A$2:$A$27</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'percent change'!$P$2:$P$27</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Year</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="6.804428502432081"/>
+          <min val="-20.55297289021944"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>% vs central</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart17.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>SC  ·  W-M L-M  ·  Res20%+contract  ·  DC series NSW  ·  Netback</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'percent change'!Q1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'percent change'!$A$2:$A$27</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'percent change'!$Q$2:$Q$27</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Year</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="10.49938730093463"/>
+          <min val="-17.75961406819361"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>% vs central</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart18.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>SC  ·  W-M L-M  ·  Res20%  ·  DC series NSW  ·  Netback</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'percent change'!R1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'percent change'!$A$2:$A$27</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'percent change'!$R$2:$R$27</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Year</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="21.04672645786252"/>
+          <min val="0"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>% vs central</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="2"/>
@@ -1415,6 +2487,839 @@
     <legend>
       <legendPos val="r"/>
     </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Acc  ·  W-M L-M  ·  Netback</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'percent change'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'percent change'!$A$2:$A$27</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'percent change'!$C$2:$C$27</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Year</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="0"/>
+          <min val="-23.41393780692444"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>% vs central</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>SG  ·  W-M L-M  ·  Netback</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'percent change'!D1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'percent change'!$A$2:$A$27</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'percent change'!$D$2:$D$27</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Year</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="54.59209976168378"/>
+          <min val="0"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>% vs central</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>SC  ·  W-M L-L  ·  Netback</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'percent change'!E1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'percent change'!$A$2:$A$27</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'percent change'!$E$2:$E$27</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Year</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="0"/>
+          <min val="-28.06269185567489"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>% vs central</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>SC  ·  W-M L-H  ·  Netback</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'percent change'!F1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'percent change'!$A$2:$A$27</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'percent change'!$F$2:$F$27</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Year</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="55.36705390895715"/>
+          <min val="0"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>% vs central</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>SC  ·  W-L L-M  ·  Netback</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'percent change'!G1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'percent change'!$A$2:$A$27</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'percent change'!$G$2:$G$27</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Year</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="18.31120174232388"/>
+          <min val="0"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>% vs central</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>SC  ·  W-H L-M  ·  Netback</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'percent change'!H1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'percent change'!$A$2:$A$27</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'percent change'!$H$2:$H$27</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Year</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="5.675792059208939"/>
+          <min val="-2.758179777732517"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>% vs central</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>SC  ·  W-M L-M  ·  Dunk27  ·  Netback</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'percent change'!I1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'percent change'!$A$2:$A$27</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'percent change'!$I$2:$I$27</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Year</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="0.4077645643328687"/>
+          <min val="0"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>% vs central</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
@@ -1467,6 +3372,363 @@
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="4" name="Chart 4"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>34</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="5" name="Chart 5"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>34</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="6" name="Chart 6"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>51</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="7" name="Chart 7"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>51</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="8" name="Chart 8"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId8"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>68</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="9" name="Chart 9"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>68</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="10" name="Chart 10"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId10"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>85</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="11" name="Chart 11"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId11"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>85</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="12" name="Chart 12"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId12"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>102</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="13" name="Chart 13"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId13"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>102</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="14" name="Chart 14"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId14"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>119</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="15" name="Chart 15"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId15"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>10</col>
+      <colOff>0</colOff>
+      <row>119</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="16" name="Chart 16"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId16"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -4882,4 +7144,18 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Bound every chart axis on a 0.5 grid
The axes were left to autoscale, so the tick labels came out at whatever
precision the renderer picked off the data. Each y-axis is now bounded
explicitly, snapped onto a 0.5 grid and formatted to one decimal.

Snapped OUTWARD rather than to the nearest: rounding a max of 21.03 down to 21.0
would put the peak of the series on the frame. The bound moves away from the
data, never into it, so no point is ever clipped to tidy an axis.

span_zero replaces the panels' hand-computed y_range and now covers the combined
percent-change chart too. The levels chart is deliberately left out of it -- a
$/GJ series in the teens forced to start at zero sits squashed in the top of the
frame.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018pSRAMaSP6de6HFGRLmysE
</commit_message>
<xml_diff>
--- a/output/domestic_price_summary.xlsx
+++ b/output/domestic_price_summary.xlsx
@@ -3446,6 +3446,8 @@
         <c:axId val="50010002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
+          <c:max val="22.0"/>
+          <c:min val="8.0"/>
         </c:scaling>
         <c:axPos val="l"/>
         <c:majorGridlines/>
@@ -3467,7 +3469,7 @@
           </c:tx>
           <c:layout/>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.0" sourceLinked="0"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50010001"/>
         <c:crosses val="autoZero"/>
@@ -3746,7 +3748,7 @@
         <c:axId val="50100002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="71.50952316672017"/>
+          <c:max val="72.0"/>
           <c:min val="0.0"/>
         </c:scaling>
         <c:axPos val="l"/>
@@ -3769,7 +3771,7 @@
           </c:tx>
           <c:layout/>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.0" sourceLinked="0"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50100001"/>
         <c:crosses val="autoZero"/>
@@ -4044,8 +4046,8 @@
         <c:axId val="50110002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="7.709110301617583"/>
-          <c:min val="-0.7561469943685784"/>
+          <c:max val="8.0"/>
+          <c:min val="-1.0"/>
         </c:scaling>
         <c:axPos val="l"/>
         <c:majorGridlines/>
@@ -4067,7 +4069,7 @@
           </c:tx>
           <c:layout/>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.0" sourceLinked="0"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50110001"/>
         <c:crosses val="autoZero"/>
@@ -4342,8 +4344,8 @@
         <c:axId val="50120002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="22.5482665569533"/>
-          <c:min val="-0.766637447044205"/>
+          <c:max val="23.0"/>
+          <c:min val="-1.0"/>
         </c:scaling>
         <c:axPos val="l"/>
         <c:majorGridlines/>
@@ -4365,7 +4367,7 @@
           </c:tx>
           <c:layout/>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.0" sourceLinked="0"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50120001"/>
         <c:crosses val="autoZero"/>
@@ -4640,8 +4642,8 @@
         <c:axId val="50130002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="2.9160916954396265"/>
-          <c:min val="-1.5987634683005236"/>
+          <c:max val="3.0"/>
+          <c:min val="-2.0"/>
         </c:scaling>
         <c:axPos val="l"/>
         <c:majorGridlines/>
@@ -4663,7 +4665,7 @@
           </c:tx>
           <c:layout/>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.0" sourceLinked="0"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50130001"/>
         <c:crosses val="autoZero"/>
@@ -4938,8 +4940,8 @@
         <c:axId val="50140002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="9.792466076806662"/>
-          <c:min val="-2.4856514869583624"/>
+          <c:max val="10.0"/>
+          <c:min val="-2.5"/>
         </c:scaling>
         <c:axPos val="l"/>
         <c:majorGridlines/>
@@ -4961,7 +4963,7 @@
           </c:tx>
           <c:layout/>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.0" sourceLinked="0"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50140001"/>
         <c:crosses val="autoZero"/>
@@ -5236,7 +5238,7 @@
         <c:axId val="50150002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="84.8294911052738"/>
+          <c:max val="85.0"/>
           <c:min val="0.0"/>
         </c:scaling>
         <c:axPos val="l"/>
@@ -5259,7 +5261,7 @@
           </c:tx>
           <c:layout/>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.0" sourceLinked="0"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50150001"/>
         <c:crosses val="autoZero"/>
@@ -5534,8 +5536,8 @@
         <c:axId val="50160002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="6.8044285024320805"/>
-          <c:min val="-20.552972890219444"/>
+          <c:max val="7.0"/>
+          <c:min val="-21.0"/>
         </c:scaling>
         <c:axPos val="l"/>
         <c:majorGridlines/>
@@ -5557,7 +5559,7 @@
           </c:tx>
           <c:layout/>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.0" sourceLinked="0"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50160001"/>
         <c:crosses val="autoZero"/>
@@ -5832,8 +5834,8 @@
         <c:axId val="50170002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="10.499387300934625"/>
-          <c:min val="-17.759614068193606"/>
+          <c:max val="10.5"/>
+          <c:min val="-18.0"/>
         </c:scaling>
         <c:axPos val="l"/>
         <c:majorGridlines/>
@@ -5855,7 +5857,7 @@
           </c:tx>
           <c:layout/>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.0" sourceLinked="0"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50170001"/>
         <c:crosses val="autoZero"/>
@@ -6130,7 +6132,7 @@
         <c:axId val="50180002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="21.04672645786252"/>
+          <c:max val="21.5"/>
           <c:min val="0.0"/>
         </c:scaling>
         <c:axPos val="l"/>
@@ -6153,7 +6155,7 @@
           </c:tx>
           <c:layout/>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.0" sourceLinked="0"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50180001"/>
         <c:crosses val="autoZero"/>
@@ -9500,6 +9502,8 @@
         <c:axId val="50020002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
+          <c:max val="85.0"/>
+          <c:min val="-28.5"/>
         </c:scaling>
         <c:axPos val="l"/>
         <c:majorGridlines/>
@@ -9521,7 +9525,7 @@
           </c:tx>
           <c:layout/>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.0" sourceLinked="0"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50020001"/>
         <c:crosses val="autoZero"/>
@@ -9801,7 +9805,7 @@
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="0.0"/>
-          <c:min val="-23.413937806924444"/>
+          <c:min val="-23.5"/>
         </c:scaling>
         <c:axPos val="l"/>
         <c:majorGridlines/>
@@ -9823,7 +9827,7 @@
           </c:tx>
           <c:layout/>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.0" sourceLinked="0"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50030001"/>
         <c:crosses val="autoZero"/>
@@ -10098,7 +10102,7 @@
         <c:axId val="50040002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="54.59209976168378"/>
+          <c:max val="55.0"/>
           <c:min val="0.0"/>
         </c:scaling>
         <c:axPos val="l"/>
@@ -10121,7 +10125,7 @@
           </c:tx>
           <c:layout/>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.0" sourceLinked="0"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50040001"/>
         <c:crosses val="autoZero"/>
@@ -10397,7 +10401,7 @@
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="0.0"/>
-          <c:min val="-28.062691855674892"/>
+          <c:min val="-28.5"/>
         </c:scaling>
         <c:axPos val="l"/>
         <c:majorGridlines/>
@@ -10419,7 +10423,7 @@
           </c:tx>
           <c:layout/>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.0" sourceLinked="0"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50050001"/>
         <c:crosses val="autoZero"/>
@@ -10694,7 +10698,7 @@
         <c:axId val="50060002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="55.36705390895715"/>
+          <c:max val="55.5"/>
           <c:min val="0.0"/>
         </c:scaling>
         <c:axPos val="l"/>
@@ -10717,7 +10721,7 @@
           </c:tx>
           <c:layout/>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.0" sourceLinked="0"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50060001"/>
         <c:crosses val="autoZero"/>
@@ -10992,7 +10996,7 @@
         <c:axId val="50070002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="18.31120174232388"/>
+          <c:max val="18.5"/>
           <c:min val="0.0"/>
         </c:scaling>
         <c:axPos val="l"/>
@@ -11015,7 +11019,7 @@
           </c:tx>
           <c:layout/>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.0" sourceLinked="0"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50070001"/>
         <c:crosses val="autoZero"/>
@@ -11290,8 +11294,8 @@
         <c:axId val="50080002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="5.6757920592089395"/>
-          <c:min val="-2.7581797777325168"/>
+          <c:max val="6.0"/>
+          <c:min val="-3.0"/>
         </c:scaling>
         <c:axPos val="l"/>
         <c:majorGridlines/>
@@ -11313,7 +11317,7 @@
           </c:tx>
           <c:layout/>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.0" sourceLinked="0"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50080001"/>
         <c:crosses val="autoZero"/>
@@ -11588,7 +11592,7 @@
         <c:axId val="50090002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="0.4077645643328687"/>
+          <c:max val="0.5"/>
           <c:min val="0.0"/>
         </c:scaling>
         <c:axPos val="l"/>
@@ -11611,7 +11615,7 @@
           </c:tx>
           <c:layout/>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.0" sourceLinked="0"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50090001"/>
         <c:crosses val="autoZero"/>

</xml_diff>

<commit_message>
Say which contract rule a reservation run used, in words
short_key labelled the contract-BREAKING run 'Res20%+contract'. 'incl' in the key
is short for "including contracted volume" -- the reservation overrides the SPAs
-- but '+contract' reads as the opposite, and sitting next to a plain 'Res20%'
for the run that actually respects contracts it was exactly backwards. Both
halves of the pair now name their rule: 'uncontracted only' / 'breaks contracts'.

Affects the dashboard dropdown and the price summary workbook, which are the only
two callers.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018pSRAMaSP6de6HFGRLmysE
</commit_message>
<xml_diff>
--- a/output/domestic_price_summary.xlsx
+++ b/output/domestic_price_summary.xlsx
@@ -48,7 +48,7 @@
     <t>SC  ·  W-M L-M  ·  GSOO exp  ·  Netback</t>
   </si>
   <si>
-    <t>SC  ·  W-M L-M  ·  Res20%  ·  Netback</t>
+    <t>SC  ·  W-M L-M  ·  Res20% uncontracted only  ·  Netback</t>
   </si>
   <si>
     <t>SC  ·  W-M L-M  ·  DC series NSW  ·  Netback</t>
@@ -60,13 +60,13 @@
     <t>SC  ·  W-M L-M  ·  DC series NSW  ·  No imports  ·  Netback</t>
   </si>
   <si>
-    <t>SC  ·  W-M L-M  ·  Res20%+contract  ·  Netback</t>
+    <t>SC  ·  W-M L-M  ·  Res20% breaks contracts  ·  Netback</t>
   </si>
   <si>
-    <t>SC  ·  W-M L-M  ·  Res20%+contract  ·  DC series NSW  ·  Netback</t>
+    <t>SC  ·  W-M L-M  ·  Res20% breaks contracts  ·  DC series NSW  ·  Netback</t>
   </si>
   <si>
-    <t>SC  ·  W-M L-M  ·  Res20%  ·  DC series NSW  ·  Netback</t>
+    <t>SC  ·  W-M L-M  ·  Res20% uncontracted only  ·  DC series NSW  ·  Netback</t>
   </si>
   <si>
     <t>Year</t>
@@ -2071,7 +2071,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>SC  ·  W-M L-M  ·  Res20%  ·  Netback</c:v>
+                  <c:v>SC  ·  W-M L-M  ·  Res20% uncontracted only  ·  Netback</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2839,7 +2839,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>SC  ·  W-M L-M  ·  Res20%+contract  ·  Netback</c:v>
+                  <c:v>SC  ·  W-M L-M  ·  Res20% breaks contracts  ·  Netback</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -3031,7 +3031,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>SC  ·  W-M L-M  ·  Res20%+contract  ·  DC series NSW  ·  Netback</c:v>
+                  <c:v>SC  ·  W-M L-M  ·  Res20% breaks contracts  ·  DC series NSW  ·  Netback</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -3223,7 +3223,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>SC  ·  W-M L-M  ·  Res20%  ·  DC series NSW  ·  Netback</c:v>
+                  <c:v>SC  ·  W-M L-M  ·  Res20% uncontracted only  ·  DC series NSW  ·  Netback</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -4101,7 +4101,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>SC  ·  W-M L-M  ·  Res20%  ·  Netback</a:t>
+              <a:t>SC  ·  W-M L-M  ·  Res20% uncontracted only  ·  Netback</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -4121,7 +4121,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>SC  ·  W-M L-M  ·  Res20%  ·  Netback</c:v>
+                  <c:v>SC  ·  W-M L-M  ·  Res20% uncontracted only  ·  Netback</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -5293,7 +5293,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>SC  ·  W-M L-M  ·  Res20%+contract  ·  Netback</a:t>
+              <a:t>SC  ·  W-M L-M  ·  Res20% breaks contracts  ·  Netback</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -5313,7 +5313,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>SC  ·  W-M L-M  ·  Res20%+contract  ·  Netback</c:v>
+                  <c:v>SC  ·  W-M L-M  ·  Res20% breaks contracts  ·  Netback</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -5591,7 +5591,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>SC  ·  W-M L-M  ·  Res20%+contract  ·  DC series NSW  ·  Netback</a:t>
+              <a:t>SC  ·  W-M L-M  ·  Res20% breaks contracts  ·  DC series NSW  ·  Netback</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -5611,7 +5611,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>SC  ·  W-M L-M  ·  Res20%+contract  ·  DC series NSW  ·  Netback</c:v>
+                  <c:v>SC  ·  W-M L-M  ·  Res20% breaks contracts  ·  DC series NSW  ·  Netback</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -5889,7 +5889,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>SC  ·  W-M L-M  ·  Res20%  ·  DC series NSW  ·  Netback</a:t>
+              <a:t>SC  ·  W-M L-M  ·  Res20% uncontracted only  ·  DC series NSW  ·  Netback</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -5909,7 +5909,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>SC  ·  W-M L-M  ·  Res20%  ·  DC series NSW  ·  Netback</c:v>
+                  <c:v>SC  ·  W-M L-M  ·  Res20% uncontracted only  ·  DC series NSW  ·  Netback</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -8127,7 +8127,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>SC  ·  W-M L-M  ·  Res20%  ·  Netback</c:v>
+                  <c:v>SC  ·  W-M L-M  ·  Res20% uncontracted only  ·  Netback</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -8895,7 +8895,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>SC  ·  W-M L-M  ·  Res20%+contract  ·  Netback</c:v>
+                  <c:v>SC  ·  W-M L-M  ·  Res20% breaks contracts  ·  Netback</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -9087,7 +9087,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>SC  ·  W-M L-M  ·  Res20%+contract  ·  DC series NSW  ·  Netback</c:v>
+                  <c:v>SC  ·  W-M L-M  ·  Res20% breaks contracts  ·  DC series NSW  ·  Netback</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -9279,7 +9279,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>SC  ·  W-M L-M  ·  Res20%  ·  DC series NSW  ·  Netback</c:v>
+                  <c:v>SC  ·  W-M L-M  ·  Res20% uncontracted only  ·  DC series NSW  ·  Netback</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>

</xml_diff>

<commit_message>
Regenerate the price workbook after costing the reserved tranche
Only the four reservation columns move. The contract-respecting 20% run goes from
+3.88% to +4.35% against central -- costing the tranche makes a reservation
slightly LESS attractive, which is the expected direction once the phantom saving
is gone.

Recorded because it refutes the prediction that motivated the change: the capacity
MIP still declines the Vopak Victoria FSRU in every reservation run, so the
uncosted tranche was not what suppressed it.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018pSRAMaSP6de6HFGRLmysE
</commit_message>
<xml_diff>
--- a/output/domestic_price_summary.xlsx
+++ b/output/domestic_price_summary.xlsx
@@ -2173,37 +2173,37 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="26"/>
                 <c:pt idx="0">
-                  <c:v>10.80988597869873</c:v>
+                  <c:v>10.89763832092285</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>11.08655166625977</c:v>
+                  <c:v>11.17911243438721</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>11.33691310882568</c:v>
+                  <c:v>11.4369945526123</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>11.57836532592773</c:v>
+                  <c:v>11.68558597564697</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>12.3137035369873</c:v>
+                  <c:v>12.70683670043945</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>12.26032733917236</c:v>
+                  <c:v>12.33250141143799</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>12.41421699523926</c:v>
+                  <c:v>12.50737571716309</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>12.60287666320801</c:v>
+                  <c:v>12.69899463653564</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>12.79858112335205</c:v>
+                  <c:v>12.8897762298584</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>13.01634979248047</c:v>
+                  <c:v>13.10569000244141</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>13.4949893951416</c:v>
+                  <c:v>13.70723533630371</c:v>
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>10.9560375213623</c:v>
@@ -4223,37 +4223,37 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="26"/>
                 <c:pt idx="0">
-                  <c:v>0.2020397216015546</c:v>
+                  <c:v>1.015458447620654</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-0.09801918068477189</c:v>
+                  <c:v>0.7360547821174457</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.216009250385607</c:v>
+                  <c:v>1.100708885994872</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.84206287957589</c:v>
+                  <c:v>2.785164245210203</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.07451419288433403</c:v>
+                  <c:v>3.26954079291657</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.97114120637245</c:v>
+                  <c:v>1.565537933357675</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-0.6895220570003913</c:v>
+                  <c:v>0.05572326957656859</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>5.834419034359839</c:v>
+                  <c:v>6.641583155515418</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>8.071366495559996</c:v>
+                  <c:v>8.841419025825781</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>10.04846407339621</c:v>
+                  <c:v>10.80380278531956</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>14.24410812793835</c:v>
+                  <c:v>16.040911929842</c:v>
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>7.649768807982493</c:v>
@@ -4344,8 +4344,8 @@
         <c:axId val="50120002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="14.5"/>
-          <c:min val="-1.0"/>
+          <c:max val="16.5"/>
+          <c:min val="0.0"/>
         </c:scaling>
         <c:axPos val="l"/>
         <c:majorGridlines/>
@@ -8229,37 +8229,37 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="26"/>
                 <c:pt idx="0">
-                  <c:v>0.2020397216015546</c:v>
+                  <c:v>1.015458447620654</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-0.09801918068477189</c:v>
+                  <c:v>0.7360547821174457</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.216009250385607</c:v>
+                  <c:v>1.100708885994872</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.84206287957589</c:v>
+                  <c:v>2.785164245210203</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.07451419288433403</c:v>
+                  <c:v>3.26954079291657</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.97114120637245</c:v>
+                  <c:v>1.565537933357675</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-0.6895220570003913</c:v>
+                  <c:v>0.05572326957656859</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>5.834419034359839</c:v>
+                  <c:v>6.641583155515418</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>8.071366495559996</c:v>
+                  <c:v>8.841419025825781</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>10.04846407339621</c:v>
+                  <c:v>10.80380278531956</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>14.24410812793835</c:v>
+                  <c:v>16.040911929842</c:v>
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>7.649768807982493</c:v>
@@ -12566,7 +12566,7 @@
         <v>10.78849792480469</v>
       </c>
       <c r="L2">
-        <v>10.80988597869873</v>
+        <v>10.89763832092285</v>
       </c>
       <c r="M2">
         <v>10.82431983947754</v>
@@ -12622,7 +12622,7 @@
         <v>11.09786701202393</v>
       </c>
       <c r="L3">
-        <v>11.08655166625977</v>
+        <v>11.17911243438721</v>
       </c>
       <c r="M3">
         <v>11.10275936126709</v>
@@ -12678,7 +12678,7 @@
         <v>11.31296348571777</v>
       </c>
       <c r="L4">
-        <v>11.33691310882568</v>
+        <v>11.4369945526123</v>
       </c>
       <c r="M4">
         <v>11.32342147827148</v>
@@ -12734,7 +12734,7 @@
         <v>11.36948013305664</v>
       </c>
       <c r="L5">
-        <v>11.57836532592773</v>
+        <v>11.68558597564697</v>
       </c>
       <c r="M5">
         <v>11.44236660003662</v>
@@ -12790,7 +12790,7 @@
         <v>12.26796245574951</v>
       </c>
       <c r="L6">
-        <v>12.3137035369873</v>
+        <v>12.70683670043945</v>
       </c>
       <c r="M6">
         <v>12.4367504119873</v>
@@ -12846,7 +12846,7 @@
         <v>12.05098724365234</v>
       </c>
       <c r="L7">
-        <v>12.26032733917236</v>
+        <v>12.33250141143799</v>
       </c>
       <c r="M7">
         <v>12.07330703735352</v>
@@ -12902,7 +12902,7 @@
         <v>12.41473579406738</v>
       </c>
       <c r="L8">
-        <v>12.41421699523926</v>
+        <v>12.50737571716309</v>
       </c>
       <c r="M8">
         <v>12.30055809020996</v>
@@ -12958,7 +12958,7 @@
         <v>11.824538230896</v>
       </c>
       <c r="L9">
-        <v>12.60287666320801</v>
+        <v>12.69899463653564</v>
       </c>
       <c r="M9">
         <v>11.93213081359863</v>
@@ -13014,7 +13014,7 @@
         <v>11.75459957122803</v>
       </c>
       <c r="L10">
-        <v>12.79858112335205</v>
+        <v>12.8897762298584</v>
       </c>
       <c r="M10">
         <v>11.88990116119385</v>
@@ -13070,7 +13070,7 @@
         <v>11.74276924133301</v>
       </c>
       <c r="L11">
-        <v>13.01634979248047</v>
+        <v>13.10569000244141</v>
       </c>
       <c r="M11">
         <v>11.92905712127686</v>
@@ -13126,7 +13126,7 @@
         <v>11.72309684753418</v>
       </c>
       <c r="L12">
-        <v>13.4949893951416</v>
+        <v>13.70723533630371</v>
       </c>
       <c r="M12">
         <v>12.01075172424316</v>
@@ -14089,7 +14089,7 @@
         <v>0.003783548494662448</v>
       </c>
       <c r="L2">
-        <v>0.2020397216015546</v>
+        <v>1.015458447620654</v>
       </c>
       <c r="M2">
         <v>0.3358341292339917</v>
@@ -14145,7 +14145,7 @@
         <v>0.003944485703510914</v>
       </c>
       <c r="L3">
-        <v>-0.09801918068477189</v>
+        <v>0.7360547821174457</v>
       </c>
       <c r="M3">
         <v>0.04802991415457925</v>
@@ -14201,7 +14201,7 @@
         <v>0.004299446501065951</v>
       </c>
       <c r="L4">
-        <v>0.216009250385607</v>
+        <v>1.100708885994872</v>
       </c>
       <c r="M4">
         <v>0.09674597656110784</v>
@@ -14257,7 +14257,7 @@
         <v>0.00473106734222295</v>
       </c>
       <c r="L5">
-        <v>1.84206287957589</v>
+        <v>2.785164245210203</v>
       </c>
       <c r="M5">
         <v>0.6458326342985599</v>
@@ -14313,7 +14313,7 @@
         <v>-0.2972274581778067</v>
       </c>
       <c r="L6">
-        <v>0.07451419288433403</v>
+        <v>3.26954079291657</v>
       </c>
       <c r="M6">
         <v>1.074526593831759</v>
@@ -14369,7 +14369,7 @@
         <v>-0.75289990282148</v>
       </c>
       <c r="L7">
-        <v>0.97114120637245</v>
+        <v>1.565537933357675</v>
       </c>
       <c r="M7">
         <v>-0.5690830291644744</v>
@@ -14425,7 +14425,7 @@
         <v>-0.6853718025302769</v>
       </c>
       <c r="L8">
-        <v>-0.6895220570003913</v>
+        <v>0.05572326957656859</v>
       </c>
       <c r="M8">
         <v>-1.598763468300524</v>
@@ -14481,7 +14481,7 @@
         <v>-0.7017867857237792</v>
       </c>
       <c r="L9">
-        <v>5.834419034359839</v>
+        <v>6.641583155515418</v>
       </c>
       <c r="M9">
         <v>0.201736972148292</v>
@@ -14537,7 +14537,7 @@
         <v>-0.7440257613474111</v>
       </c>
       <c r="L10">
-        <v>8.071366495559996</v>
+        <v>8.841419025825781</v>
       </c>
       <c r="M10">
         <v>0.3984624235302547</v>
@@ -14593,7 +14593,7 @@
         <v>-0.7191924326155674</v>
       </c>
       <c r="L11">
-        <v>10.04846407339621</v>
+        <v>10.80380278531956</v>
       </c>
       <c r="M11">
         <v>0.8558032758704481</v>
@@ -14649,7 +14649,7 @@
         <v>-0.7561469943685784</v>
       </c>
       <c r="L12">
-        <v>14.24410812793835</v>
+        <v>16.040911929842</v>
       </c>
       <c r="M12">
         <v>1.679043866181562</v>

</xml_diff>